<commit_message>
Perbarui konten pajak UMKM sesuai PP 20/2026
PP 20/2026 mengubah PP 55/2022: PPh Final 0,5% kini hanya untuk orang
pribadi, PT perorangan, dan koperasi; tanpa batas waktu untuk orang
pribadi dan PT perorangan; CV, firma, dan PT biasa tidak lagi berhak
kecuali selama masa transisi; omzet suami-istri dan PT perorangan
digabung untuk batas Rp4,8 miliar. Batas omzet bebas pajak Rp500 juta
bagi orang pribadi tetap berlaku.

- Kalkulator pajak UMKM: pilihan "Badan (PT, CV, firma, koperasi)"
  diganti "PT perorangan atau koperasi", catatan hasil diperbarui
- Artikel pajak UMKM: siapa yang berhak, tabel jangka waktu baru,
  contoh PT perorangan, aturan penggabungan omzet, sumber hukum
- Template pembukuan: catatan dan pilihan jenis wajib pajak

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EBT8K2zktY7qYZgeyqq2GY
</commit_message>
<xml_diff>
--- a/assets/template-pembukuan-umkm.xlsx
+++ b/assets/template-pembukuan-umkm.xlsx
@@ -569,7 +569,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>PPh Final 0,5% mengikuti PP 55/2022: orang pribadi tidak dikenai pajak atas omzet sampai Rp500 juta setahun.</t>
+          <t>PPh Final 0,5% mengikuti PP 55/2022 sebagaimana diubah PP 20/2026: orang pribadi tidak dikenai pajak atas omzet sampai Rp500 juta setahun.</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PP 55/2022: Rp500 juta hanya untuk orang pribadi, badan Rp0.</t>
+          <t>Rp500 juta hanya untuk orang pribadi; PT perorangan dan koperasi Rp0.</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>PP 55/2022 Pasal 57. Cek perubahan aturan di pajak.go.id.</t>
+          <t>PP 55/2022 jo. PP 20/2026. Cek perubahan aturan di pajak.go.id.</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Orang pribadi,Badan"</formula1>
+      <formula1>"Orang pribadi,PT perorangan/koperasi"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>